<commit_message>
Clean synthetic workbook metadata
</commit_message>
<xml_diff>
--- a/google-apps-script/aff-partners-info/anonymized_table.xlsx
+++ b/google-apps-script/aff-partners-info/anonymized_table.xlsx
@@ -8,10 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="Synthetic Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Hidden Sheet" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="synthetic_range">'Synthetic Summary'!A1:D3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Synthetic Summary'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -126,21 +124,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Automation Bot</author>
-  </authors>
-  <commentList>
-    <comment ref="E2" authorId="0" shapeId="0">
-      <text>
-        <t>Synthetic data only</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -432,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,11 +461,6 @@
           <t>Approved</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>note</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -503,28 +481,6 @@
       <c r="D3" t="inlineStr">
         <is>
           <t>Pending</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>hidden</t>
         </is>
       </c>
     </row>

</xml_diff>